<commit_message>
WIP：每小时保存全部进度 2026-09-19 02:51:18 -04:00
</commit_message>
<xml_diff>
--- a/data/MessageLimiter.xlsx
+++ b/data/MessageLimiter.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1082,6 +1082,104 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>216</v>
+      </c>
+      <c r="B52" t="n">
+        <v>5</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>217</v>
+      </c>
+      <c r="B53" t="n">
+        <v>5</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>218</v>
+      </c>
+      <c r="B54" t="n">
+        <v>5</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>219</v>
+      </c>
+      <c r="B55" t="n">
+        <v>5</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>221</v>
+      </c>
+      <c r="B56" t="n">
+        <v>10</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>222</v>
+      </c>
+      <c r="B57" t="n">
+        <v>10</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>223</v>
+      </c>
+      <c r="B58" t="n">
+        <v>5</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>